<commit_message>
Finalize audited Section 32 report package
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SECTION32_BEST_OF_BEST_TOURNAMENT_20260806/FINAL_CHAMPION/SECTION32_BEST_OF_BEST_SOURCE_LINEAGE_20260806.xlsx
+++ b/SECTION32_BEST_OF_BEST_TOURNAMENT_20260806/FINAL_CHAMPION/SECTION32_BEST_OF_BEST_SOURCE_LINEAGE_20260806.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Conflict Register" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cell Lineage'!$A$1:$F$167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cell Lineage'!$A$1:$F$166</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -689,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F167"/>
+  <dimension ref="A1:F166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -745,7 +745,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>TRACT 1 estimated owner: Adolf Bollenbach, or his unlocated successors and assigns (65.000000 NMA)</t>
+          <t>TRACT 1 estimated owner: Unresolved successors of Adolf Bollenbach (last proved record owner, WD 10/255, 01/31/1910) — chain gap remains unresolved (65.000000 NMA)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 65.000000 NMA residual vests in last traced record owner (WD 10/255); no chain-out located. Current status is not confirmed through the report effective date.</t>
+          <t>ASSUMED: 65.000000 NMA residual vests in last traced record owner (WD 10/255); no chain-out located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: WD 10/255. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>TRACT 1 estimated owner: C. B. Crook, Jr. (8.000000 NMA)</t>
+          <t>TRACT 1 estimated owner: C. B. Crook, Jr. — last located record owner; no later conveyance located; current status not confirmed (8.000000 NMA)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>TRACT 1 estimated owner: Carole Faye Hanks (8.000000 NMA)</t>
+          <t>TRACT 1 estimated owner: Carole Faye Hanks — last located record owner; no later conveyance located; current status not confirmed (8.000000 NMA)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>TRACT 1 estimated owner: Doris Marie Lenderman (8.000000 NMA)</t>
+          <t>TRACT 1 estimated owner: Doris Marie Lenderman — last located record owner; no later conveyance located; current status not confirmed (8.000000 NMA)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>TRACT 1 estimated owner: F. L. Randel and J. L. Randel, share and share alike (Wichita Falls, TX) (1.500000 NMA)</t>
+          <t>TRACT 1 estimated owner: F. L. Randel and J. L. Randel, share and share alike (Wichita Falls, TX) — last located record owner; no later conveyance located; current status not confirmed (1.500000 NMA)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 92/47; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 92/47; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 92/47. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>TRACT 1 estimated owner: Five issue of Charlie B. Crook (collective row - chained out) (0.000000 NMA)</t>
+          <t>TRACT 1 estimated owner: Great Western (entity as shown on the reviewed face, img 1558) — last located record owner; no later conveyance located; current status not confirmed (10.000000 NMA)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Chained out: distributed individually per DECR 845/149-153 and 845/152 clause (h); retained at 0 NMA for audit. Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 367/632; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 367/632. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>TRACT 1 estimated owner: Great Western (entity as shown on the reviewed face, img 1558) (10.000000 NMA)</t>
+          <t>TRACT 1 estimated owner: Ina Bell Bryan — last located record owner; no later conveyance located; current status not confirmed (8.000000 NMA)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 367/632; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>TRACT 1 estimated owner: Ina Bell Bryan (8.000000 NMA)</t>
+          <t>TRACT 1 estimated owner: Jean Jenkins Shearer, Florence Jenkins Chunn and William Rundell Jenkins, JTWROS — last located record owner; no later conveyance located; current status not confirmed (2.000000 NMA)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 250/26; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 250/26. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>TRACT 1 estimated owner: Jean Jenkins Shearer, Florence Jenkins Chunn and William Rundell Jenkins, JTWROS (2.000000 NMA)</t>
+          <t>TRACT 1 estimated owner: Mary Joyce Higgenbotham — last located record owner; no later conveyance located; current status not confirmed (8.000000 NMA)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 250/26; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>TRACT 1 estimated owner: Mary Joyce Higgenbotham (8.000000 NMA)</t>
+          <t>TRACT 1 estimated owner: Unresolved probate beneficiaries under Decree 83/259 (Estate of Ellen W. Crook) — individual allocations not stated on the decree face (40.000000 NMA)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>ASSUMED: 40.000000 NMA vests collectively per decree; individual allocations not stated on the face. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>TRACT 1 estimated owner: Beneficiaries of Ellen W. Crook (13 named, DECR 83/259) (40.000000 NMA)</t>
+          <t>TRACT 1 estimated owner: Unresolved record owner — grantee of the F. L. Randel 1.5-acre deed (img 1794); grantee name not read from the face (1.500000 NMA)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 40.000000 NMA vests collectively per decree; individual allocations not stated on the face. Current status is not confirmed through the report effective date.</t>
+          <t>ASSUMED: holds 1.500000 NMA per the recorded deed; grantee name not extracted from the face. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1092,12 +1092,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>B17:G17</t>
+          <t>B23:G23</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>TRACT 1 estimated owner: Grantee of the F. L. Randel 1.5-acre deed (img 1794) (1.500000 NMA)</t>
+          <t>TRACT 2 estimated owner: B. E. Maddoux (stipulated residual) — last located record owner; no later conveyance located; current status not confirmed (10.000000 NMA)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: holds 1.500000 NMA per the recorded deed; grantee name not extracted from the face. Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: STIPULATION (RECORDED QUANTUM) 153/161-162. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1124,12 +1124,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>B22:G22</t>
+          <t>B24:G24</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: B. E. Maddoux (stipulated residual) (10.000000 NMA)</t>
+          <t>TRACT 2 estimated owner: D. H. Maddoux (stipulated residual) — last located record owner; no later conveyance located; current status not confirmed (10.000000 NMA)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: STIPULATION (RECORDED QUANTUM) 153/161-162. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>B23:G23</t>
+          <t>B25:G25</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: D. H. Maddoux (stipulated residual) (10.000000 NMA)</t>
+          <t>TRACT 2 estimated owner: E. C. (E. G.) Sanditen — last located record owner; no later conveyance located; current status not confirmed (7.500000 NMA)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 85/365 corr. 87/174; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/365 corr. 87/174. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1188,12 +1188,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>B24:G24</t>
+          <t>B26:G26</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: E. C. (E. G.) Sanditen (7.500000 NMA)</t>
+          <t>TRACT 2 estimated owner: Edna Mae Walker Revocable Trust dtd 05/21/1981 — last located record owner; no later conveyance located; current status not confirmed (0.416666 NMA)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/365 corr. 87/174; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 1287/42; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1287/42. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1220,12 +1220,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>B25:G25</t>
+          <t>B27:G27</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: Edna Mae Walker Revocable Trust dtd 05/21/1981 (0.416666 NMA)</t>
+          <t>TRACT 2 estimated owner: First National Bank &amp; Trust Co. of Tulsa, Trustee u/w Mylon C. Jacobs, Sr. — last located record owner; no later conveyance located; current status not confirmed (0.250000 NMA)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1287/42; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR 312/700-704; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 312/700-704. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1252,12 +1252,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>B26:G26</t>
+          <t>B28:G28</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: First National Bank &amp; Trust Co. of Tulsa, Trustee u/w Mylon C. Jacobs, Sr. (0.250000 NMA)</t>
+          <t>TRACT 2 estimated owner: George T. Harrison, Jr. and Renata Harrison — last located record owner; no later conveyance located; current status not confirmed (0.100000 NMA)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 312/700-704; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/424; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/424. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1284,12 +1284,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>B27:G27</t>
+          <t>B29:G29</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: George T. Harrison, Jr. and Renata Harrison (0.100000 NMA)</t>
+          <t>TRACT 2 estimated owner: Herman Sanditen — last located record owner; no later conveyance located; current status not confirmed (7.500000 NMA)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/424; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 85/363; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/363. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1316,12 +1316,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>B28:G28</t>
+          <t>B30:G30</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: Herman Sanditen (7.500000 NMA)</t>
+          <t>TRACT 2 estimated owner: J. F. Costello (Lindsay, OK) — last located record owner; no later conveyance located; current status not confirmed (5.000000 NMA)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/363; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/245; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/245. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1348,12 +1348,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>B29:G29</t>
+          <t>B31:G31</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: J. F. Costello (Lindsay, OK) (5.000000 NMA)</t>
+          <t>TRACT 2 estimated owner: Jack V. Walker Revocable Trust dtd 05/21/1981 — last located record owner; no later conveyance located; current status not confirmed (0.416666 NMA)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/245; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 1287/42; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1287/42. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1380,12 +1380,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>B30:G30</t>
+          <t>B32:G32</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: Jack V. Walker Revocable Trust dtd 05/21/1981 (0.416666 NMA)</t>
+          <t>TRACT 2 estimated owner: James M. Murray, Jr. — last located record owner; no later conveyance located; current status not confirmed (0.200000 NMA)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1287/42; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/428; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/428. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1412,12 +1412,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>B31:G31</t>
+          <t>B33:G33</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: James M. Murray, Jr. (0.200000 NMA)</t>
+          <t>TRACT 2 estimated owner: John Holbrook — last located record owner; no later conveyance located; current status not confirmed (0.100000 NMA)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/428; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/426; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/426. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1444,12 +1444,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>B32:G32</t>
+          <t>B34:G34</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: John Holbrook (0.100000 NMA)</t>
+          <t>TRACT 2 estimated owner: Julius Sanditen — last located record owner; no later conveyance located; current status not confirmed (7.500000 NMA)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/426; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 85/364; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/364. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1476,12 +1476,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>B33:G33</t>
+          <t>B35:G35</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: Julius Sanditen (7.500000 NMA)</t>
+          <t>TRACT 2 estimated owner: Kershaw Properties — last located record owner; no later conveyance located; current status not confirmed (3.375000 NMA)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/364; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: ORDER 311/817-828. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1508,12 +1508,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>B34:G34</t>
+          <t>B36:G36</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: Kershaw Properties (3.375000 NMA)</t>
+          <t>TRACT 2 estimated owner: Louis Fenster — last located record owner; no later conveyance located; current status not confirmed (4.000000 NMA)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 85/366; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/366. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1540,12 +1540,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>B35:G35</t>
+          <t>B37:G37</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: Louis Fenster (4.000000 NMA)</t>
+          <t>TRACT 2 estimated owner: Mathew Keck (Chicago) — last located record owner; no later conveyance located; current status not confirmed (1.000000 NMA)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/366; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 88/172; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 88/172. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1572,12 +1572,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>B36:G36</t>
+          <t>B38:G38</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: Mathew Keck (Chicago) (1.000000 NMA)</t>
+          <t>TRACT 2 estimated owner: Robert A. Gannaway — last located record owner; no later conveyance located; current status not confirmed (3.375000 NMA)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 88/172; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: ORDER 311/817-828. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>B37:G37</t>
+          <t>B39:G39</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: Robert A. Gannaway (3.375000 NMA)</t>
+          <t>TRACT 2 estimated owner: Robert R. Lockwood, Jr. — last located record owner; no later conveyance located; current status not confirmed (0.250000 NMA)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1619,7 +1619,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/87; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/87. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1636,12 +1636,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>B38:G38</t>
+          <t>B40:G40</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: Robert R. Lockwood, Jr. (0.250000 NMA)</t>
+          <t>TRACT 2 estimated owner: Sara M. Smith — last located record owner; no later conveyance located; current status not confirmed (0.100000 NMA)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/87; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/422; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/422. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>B39:G39</t>
+          <t>B41:G41</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: Sara M. Smith (0.100000 NMA)</t>
+          <t>TRACT 2 estimated owner: Untraced successor interest in the Farrar N/2 NW/4 fee — connecting instrument not located (12.166667 NMA)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/422; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>ASSUMED: 12.166667 NMA carried in the Farrar fee chain; connecting instrument not located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1700,12 +1700,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>B40:G40</t>
+          <t>B42:G42</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: Successors of the Farrar NW/4 fee (Farrar-to-Maddoux chain) (12.166667 NMA)</t>
+          <t>TRACT 2 estimated owner: Unresolved successors of Maurice Sanditen (index reference 92/468; later family instruments unread) (6.750000 NMA)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 12.166667 NMA carried in the Farrar fee chain; connecting instrument not located. Current status is not confirmed through the report effective date.</t>
+          <t>ASSUMED: 6.750000 NMA per 92/468 (index) and later family instruments not read. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: 92/468. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1732,12 +1732,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>B41:G41</t>
+          <t>B47:G47</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>TRACT 2 estimated owner: Maurice Sanditen, or his successors and assigns (6.750000 NMA)</t>
+          <t>TRACT 3 estimated owner: Claud B. Hamill — last located record owner; no later conveyance located; current status not confirmed (40.000000 NMA)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 6.750000 NMA per 92/468 (index) and later family instruments not read. Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 86/21; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 86/21. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1764,12 +1764,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>B46:G46</t>
+          <t>B48:G48</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>TRACT 3 estimated owner: Claud B. Hamill (40.000000 NMA)</t>
+          <t>TRACT 3 estimated owner: Unresolved successors of G. B. and Ola Keathley — residue exposed by Decree P-76-78 (13.333333 NMA)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 86/21; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>ASSUMED: 13.333333 NMA residue exposed by DECR P-76-78 vests in untraced Keathley successors. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1796,12 +1796,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>B47:G47</t>
+          <t>B49:G49</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>TRACT 3 estimated owner: Successors of G. B. and Ola Keathley (13.333333 NMA)</t>
+          <t>TRACT 3 estimated owner: J. A. Brescian — last located record owner; no later conveyance located; current status not confirmed (10.000000 NMA)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 13.333333 NMA residue exposed by DECR P-76-78 vests in untraced Keathley successors. Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 85/36; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/36. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -1828,12 +1828,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>B48:G48</t>
+          <t>B50:G50</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>TRACT 3 estimated owner: J. A. Brescian (10.000000 NMA)</t>
+          <t>TRACT 3 estimated owner: Leo Keathley and La Wanda Keathley, H/W — last located record owner; no later conveyance located; current status not confirmed (2.222222 NMA)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/36; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR P-76-78, pages 349-350 (images 1546-1550); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR P-76-78, pages 349-350 (images 1546-1550). Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1860,12 +1860,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>B49:G49</t>
+          <t>B51:G51</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>TRACT 3 estimated owner: Leo Keathley and La Wanda Keathley, H/W (2.222222 NMA)</t>
+          <t>TRACT 3 estimated owner: Milton Keathley and Inez Keathley, H/W — last located record owner; no later conveyance located; current status not confirmed (2.222222 NMA)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR P-76-78, pages 349-350 (images 1546-1550); EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR P-76-78, pages 349-350 (images 1546-1550); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR P-76-78, pages 349-350 (images 1546-1550). Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1892,12 +1892,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>B50:G50</t>
+          <t>B52:G52</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>TRACT 3 estimated owner: Milton Keathley and Inez Keathley, H/W (2.222222 NMA)</t>
+          <t>TRACT 3 estimated owner: Slemp Oil Company — last located record owner; no later conveyance located; current status not confirmed (10.000000 NMA)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR P-76-78, pages 349-350 (images 1546-1550); EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 74/63; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 74/63. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1924,12 +1924,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>B51:G51</t>
+          <t>B53:G53</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>TRACT 3 estimated owner: Slemp Oil Company (10.000000 NMA)</t>
+          <t>TRACT 3 estimated owner: T. G. Le Grand and Juanita Le Grand, H/W — last located record owner; no later conveyance located; current status not confirmed (2.222222 NMA)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 74/63; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR P-76-78, pages 349-350 (images 1546-1550); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR P-76-78, pages 349-350 (images 1546-1550). Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1956,12 +1956,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>B52:G52</t>
+          <t>B58:G58</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>TRACT 3 estimated owner: T. G. Le Grand and Juanita Le Grand, H/W (2.222222 NMA)</t>
+          <t>TRACT 4 estimated owner: B. E. Maddoux (stipulated residual) — last located record owner; no later conveyance located; current status not confirmed (10.000000 NMA)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR P-76-78, pages 349-350 (images 1546-1550); EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: STIPULATION (RECORDED QUANTUM) 153/161-162. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -1988,12 +1988,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>B57:G57</t>
+          <t>B59:G59</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: B. E. Maddoux (stipulated residual) (10.000000 NMA)</t>
+          <t>TRACT 4 estimated owner: D. H. Maddoux (stipulated residual) — last located record owner; no later conveyance located; current status not confirmed (10.000000 NMA)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: STIPULATION (RECORDED QUANTUM) 153/161-162. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2020,12 +2020,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>B58:G58</t>
+          <t>B60:G60</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: D. H. Maddoux (stipulated residual) (10.000000 NMA)</t>
+          <t>TRACT 4 estimated owner: Edna Mae Walker Revocable Trust dtd 05/21/1981 — last located record owner; no later conveyance located; current status not confirmed (0.416666 NMA)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 1287/42; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1287/42. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2052,12 +2052,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>B59:G59</t>
+          <t>B61:G61</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: Edna Mae Walker Revocable Trust dtd 05/21/1981 (0.416666 NMA)</t>
+          <t>TRACT 4 estimated owner: First National Bank &amp; Trust Co. of Tulsa, Trustee u/w Mylon C. Jacobs, Sr. — last located record owner; no later conveyance located; current status not confirmed (1.000000 NMA)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1287/42; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR 312/700-704; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 312/700-704. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2084,12 +2084,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>B60:G60</t>
+          <t>B62:G62</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: First National Bank &amp; Trust Co. of Tulsa, Trustee u/w Mylon C. Jacobs, Sr. (1.000000 NMA)</t>
+          <t>TRACT 4 estimated owner: George T. Harrison, Jr. and Renata Harrison — last located record owner; no later conveyance located; current status not confirmed (0.400000 NMA)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 312/700-704; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/424; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/424. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2116,12 +2116,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>B61:G61</t>
+          <t>B63:G63</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: George T. Harrison, Jr. and Renata Harrison (0.400000 NMA)</t>
+          <t>TRACT 4 estimated owner: Gertrude L. LaFortune, Jeanne L. Fair, Mary Ann L. Wilcox, J. A. LaFortune Jr. and Robert J. LaFortune, Co-Trustees u/w (in trust) — last located record owner; no later conveyance located; current status not confirmed (1.333334 NMA)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/424; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR 333/239-248; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 333/239-248. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2148,12 +2148,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>B62:G62</t>
+          <t>B64:G64</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: Gertrude L. LaFortune, Jeanne L. Fair, Mary Ann L. Wilcox, J. A. LaFortune Jr. and Robert J. LaFortune, Co-Trustees u/w (in trust) (1.333334 NMA)</t>
+          <t>TRACT 4 estimated owner: Helen Langer May (Palos Park, IL) — last located record owner; no later conveyance located; current status not confirmed (1.000000 NMA)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 333/239-248; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 88/174; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 88/174. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2180,12 +2180,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>B63:G63</t>
+          <t>B65:G65</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: Helen Langer May (Palos Park, IL) (1.000000 NMA)</t>
+          <t>TRACT 4 estimated owner: Jack V. Walker Revocable Trust dtd 05/21/1981 — last located record owner; no later conveyance located; current status not confirmed (0.416666 NMA)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 88/174; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 1287/42; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1287/42. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2212,12 +2212,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>B64:G64</t>
+          <t>B66:G66</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: Jack V. Walker Revocable Trust dtd 05/21/1981 (0.416666 NMA)</t>
+          <t>TRACT 4 estimated owner: James M. Murray, Jr. — last located record owner; no later conveyance located; current status not confirmed (0.800000 NMA)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1287/42; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/428; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/428. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2244,12 +2244,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>B65:G65</t>
+          <t>B67:G67</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: James M. Murray, Jr. (0.800000 NMA)</t>
+          <t>TRACT 4 estimated owner: John Holbrook — last located record owner; no later conveyance located; current status not confirmed (0.400000 NMA)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -2259,7 +2259,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/428; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/426; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/426. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2276,12 +2276,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>B66:G66</t>
+          <t>B68:G68</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: John Holbrook (0.400000 NMA)</t>
+          <t>TRACT 4 estimated owner: LaFortune Tung Oil Mill — last located record owner; no later conveyance located; current status not confirmed (1.333334 NMA)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/426; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 90/242; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 90/242. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2308,12 +2308,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>B67:G67</t>
+          <t>B69:G69</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: LaFortune Tung Oil Mill (1.333334 NMA)</t>
+          <t>TRACT 4 estimated owner: Mathew Keck (Chicago) — last located record owner; no later conveyance located; current status not confirmed (3.000000 NMA)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 90/242; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 88/172; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 88/172. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2340,12 +2340,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>B68:G68</t>
+          <t>B70:G70</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: Mathew Keck (Chicago) (3.000000 NMA)</t>
+          <t>TRACT 4 estimated owner: Robert James LaFortune — last located record owner; no later conveyance located; current status not confirmed (1.333334 NMA)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 88/172; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 90/241; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 90/241. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2372,12 +2372,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>B69:G69</t>
+          <t>B71:G71</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: Robert James LaFortune (1.333334 NMA)</t>
+          <t>TRACT 4 estimated owner: Robert R. Lockwood, Jr. — last located record owner; no later conveyance located; current status not confirmed (1.000000 NMA)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 90/241; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/87; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/87. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2404,12 +2404,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>B70:G70</t>
+          <t>B72:G72</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: Robert R. Lockwood, Jr. (1.000000 NMA)</t>
+          <t>TRACT 4 estimated owner: Sara M. Smith — last located record owner; no later conveyance located; current status not confirmed (0.400000 NMA)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/87; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/422; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/422. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2436,12 +2436,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>B71:G71</t>
+          <t>B73:G73</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: Sara M. Smith (0.400000 NMA)</t>
+          <t>TRACT 4 estimated owner: Seidenbach's (entity, 413 S. Main, Tulsa) — last located record owner; no later conveyance located; current status not confirmed (5.000000 NMA)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/422; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 90/153; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 90/153. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -2468,12 +2468,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>B72:G72</t>
+          <t>B74:G74</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: Seidenbach's (entity, 413 S. Main, Tulsa) (5.000000 NMA)</t>
+          <t>TRACT 4 estimated owner: T. D. Norris — last located record owner; no later conveyance located; current status not confirmed (5.000000 NMA)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 90/153; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/315; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/315. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2500,12 +2500,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>B73:G73</t>
+          <t>B75:G75</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: T. D. Norris (5.000000 NMA)</t>
+          <t>TRACT 4 estimated owner: The Heller Company — last located record owner; no later conveyance located; current status not confirmed (17.999999 NMA)</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/315; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 85/222; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/222. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2532,12 +2532,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>B74:G74</t>
+          <t>B76:G76</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: The Heller Company (17.999999 NMA)</t>
+          <t>TRACT 4 estimated owner: Bettye Folmar Norris — last located record owner; no later conveyance located; current status not confirmed (5.000000 NMA)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/222; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR 262/490-493 (P-71-473); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 262/490-493 (P-71-473). Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -2564,12 +2564,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>B75:G75</t>
+          <t>B77:G77</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: Bettye Folmar Norris (5.000000 NMA)</t>
+          <t>TRACT 4 estimated owner: Untraced successor interest — Stevens-to-Maddoux chain; connecting instrument not located (14.166667 NMA)</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 262/490-493 (P-71-473); EST.* Current status is not confirmed through the report effective date.</t>
+          <t>ASSUMED: 14.166667 NMA carried in the Stevens chain; connecting instrument not located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -2596,12 +2596,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>B76:G76</t>
+          <t>B82:G82</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>TRACT 4 estimated owner: Successors of the Stevens interest (Stevens-to-Maddoux chain) (14.166667 NMA)</t>
+          <t>TRACT 5 estimated owner: C. R. Bennett (812 Palace Building, Tulsa) — last located record owner; no later conveyance located; current status not confirmed (40.000000 NMA)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 14.166667 NMA carried in the Stevens chain; connecting instrument not located. Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 81/194; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 81/194. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -2628,12 +2628,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>B81:G81</t>
+          <t>B83:G83</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>TRACT 5 estimated owner: C. R. Bennett (812 Palace Building, Tulsa) (40.000000 NMA)</t>
+          <t>TRACT 5 estimated owner: Untraced successor interest — Stevens-to-LeGrand chain; connecting instrument not located (35.000000 NMA)</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 81/194; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>ASSUMED: 35.000000 NMA carried in the Stevens chain; connecting instrument not located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>B82:G82</t>
+          <t>B84:G84</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>TRACT 5 estimated owner: Successors of the Stevens interest (Stevens-to-LeGrand chain) (35.000000 NMA)</t>
+          <t>TRACT 5 estimated owner: W. F. Palmer (Wichita Falls, TX) — last located record owner; no later conveyance located; current status not confirmed (5.000000 NMA)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 35.000000 NMA carried in the Stevens chain; connecting instrument not located. Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 92/115 (previously mis-cited 92/120); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 92/115 (previously mis-cited 92/120). Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -2692,12 +2692,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>B83:G83</t>
+          <t>B89:G89</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>TRACT 5 estimated owner: W. F. Palmer (Wichita Falls, TX) (5.000000 NMA)</t>
+          <t>TRACT 6 estimated owner: Carlene Stewart — last located record owner; no later conveyance located; current status not confirmed (7.993200 NMA)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 92/115 (previously mis-cited 92/120); EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 1063/166; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1063/166. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -2724,12 +2724,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>B88:G88</t>
+          <t>B90:G90</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Carlene Stewart (7.993200 NMA)</t>
+          <t>TRACT 6 estimated owner: Unresolved successors of Cora B. Garrett and S. A. Garrett (OGL 1 lessors of record) — succession untraced (27.674000 NMA)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1063/166; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>ASSUMED: 27.674000 NMA residual vests in OGL 1 lessors of record; succession untraced. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -2756,12 +2756,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>B89:G89</t>
+          <t>B91:G91</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Cora B. Garrett and S. A. Garrett, or unlocated successors (27.674000 NMA)</t>
+          <t>TRACT 6 estimated owner: E. C. (E. G.) Sanditen — last located record owner; no later conveyance located; current status not confirmed (3.750000 NMA)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 27.674000 NMA residual vests in OGL 1 lessors of record; succession untraced. Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 85/365 corr. 87/174; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/365 corr. 87/174. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -2788,12 +2788,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>B90:G90</t>
+          <t>B92:G92</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: E. C. (E. G.) Sanditen (3.750000 NMA)</t>
+          <t>TRACT 6 estimated owner: First National Bank &amp; Trust Co. of Tulsa, Trustee u/w Mylon C. Jacobs, Sr. — last located record owner; no later conveyance located; current status not confirmed (0.500000 NMA)</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -2803,7 +2803,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/365 corr. 87/174; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR 312/700-704; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 312/700-704. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -2820,12 +2820,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>B91:G91</t>
+          <t>B93:G93</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: First National Bank &amp; Trust Co. of Tulsa, Trustee u/w Mylon C. Jacobs, Sr. (0.500000 NMA)</t>
+          <t>TRACT 6 estimated owner: George T. Harrison, Jr. and Renata Harrison — last located record owner; no later conveyance located; current status not confirmed (0.200000 NMA)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 312/700-704; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/424; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/424. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -2852,12 +2852,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>B92:G92</t>
+          <t>B94:G94</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: George T. Harrison, Jr. and Renata Harrison (0.200000 NMA)</t>
+          <t>TRACT 6 estimated owner: Herman Sanditen — last located record owner; no later conveyance located; current status not confirmed (3.750000 NMA)</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/424; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 85/363; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/363. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -2884,12 +2884,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>B93:G93</t>
+          <t>B95:G95</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Herman Sanditen (3.750000 NMA)</t>
+          <t>TRACT 6 estimated owner: J. F. Costello (Lindsay, OK) — last located record owner; no later conveyance located; current status not confirmed (5.000000 NMA)</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/363; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/244; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/244. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -2916,12 +2916,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>B94:G94</t>
+          <t>B96:G96</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: J. F. Costello (Lindsay, OK) (5.000000 NMA)</t>
+          <t>TRACT 6 estimated owner: James M. Murray, Jr. — last located record owner; no later conveyance located; current status not confirmed (0.400000 NMA)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/244; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/428; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/428. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -2948,12 +2948,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>B95:G95</t>
+          <t>B97:G97</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: James M. Murray, Jr. (0.400000 NMA)</t>
+          <t>TRACT 6 estimated owner: John Holbrook — last located record owner; no later conveyance located; current status not confirmed (0.200000 NMA)</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/428; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/426; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/426. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -2980,12 +2980,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>B96:G96</t>
+          <t>B98:G98</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: John Holbrook (0.200000 NMA)</t>
+          <t>TRACT 6 estimated owner: Joseph Ervin Godwin, III (suffix II/III uncertain) — last located record owner; no later conveyance located; current status not confirmed (0.666600 NMA)</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/426; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 1090/94; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1090/94. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -3012,12 +3012,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>B97:G97</t>
+          <t>B99:G99</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Joseph Ervin Godwin, III (suffix II/III uncertain) (0.666600 NMA)</t>
+          <t>TRACT 6 estimated owner: Julius Sanditen — last located record owner; no later conveyance located; current status not confirmed (3.750000 NMA)</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1090/94; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 85/364; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/364. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -3044,12 +3044,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>B98:G98</t>
+          <t>B100:G100</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Julius Sanditen (3.750000 NMA)</t>
+          <t>TRACT 6 estimated owner: Kershaw Properties — last located record owner; no later conveyance located; current status not confirmed (3.375000 NMA)</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -3059,7 +3059,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/364; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: ORDER 311/817-828. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -3076,12 +3076,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>B99:G99</t>
+          <t>B101:G101</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Kershaw Properties (3.375000 NMA)</t>
+          <t>TRACT 6 estimated owner: Louis Fenster — last located record owner; no later conveyance located; current status not confirmed (2.000000 NMA)</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 85/366; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/366. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -3108,12 +3108,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>B100:G100</t>
+          <t>B102:G102</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Louis Fenster (2.000000 NMA)</t>
+          <t>TRACT 6 estimated owner: Mathew Keck (Chicago) — last located record owner; no later conveyance located; current status not confirmed (2.000000 NMA)</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/366; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 88/172; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 88/172. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -3140,12 +3140,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>B101:G101</t>
+          <t>B103:G103</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Mathew Keck (Chicago) (2.000000 NMA)</t>
+          <t>TRACT 6 estimated owner: Millard E. Kuykendall — last located record owner; no later conveyance located; current status not confirmed (1.333200 NMA)</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 88/172; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 1063/164; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1063/164. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -3172,12 +3172,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>B102:G102</t>
+          <t>B104:G104</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Millard E. Kuykendall (1.333200 NMA)</t>
+          <t>TRACT 6 estimated owner: R. E. Fowler and Sue Fowler; John R. Fowler and Louise Fowler (grantees collectively per the face) — last located record owner; no later conveyance located; current status not confirmed (6.333200 NMA)</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1063/164; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 1423/148; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1423/148. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -3204,12 +3204,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>B103:G103</t>
+          <t>B105:G105</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: R. E. Fowler and Sue Fowler; John R. Fowler and Louise Fowler (grantees collectively per the face) (6.333200 NMA)</t>
+          <t>TRACT 6 estimated owner: Robert A. Gannaway — last located record owner; no later conveyance located; current status not confirmed (3.375000 NMA)</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1423/148; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: ORDER 311/817-828. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -3236,12 +3236,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>B104:G104</t>
+          <t>B106:G106</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Robert A. Gannaway (3.375000 NMA)</t>
+          <t>TRACT 6 estimated owner: Robert R. Lockwood, Jr. — last located record owner; no later conveyance located; current status not confirmed (0.500000 NMA)</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/87; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/87. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -3268,12 +3268,12 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>B105:G105</t>
+          <t>B107:G107</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Robert R. Lockwood, Jr. (0.500000 NMA)</t>
+          <t>TRACT 6 estimated owner: Royice Roberts and Pauline Roberts, JTWROS — last located record owner; no later conveyance located; current status not confirmed (1.333200 NMA)</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/87; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 1063/164; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1063/164. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -3300,12 +3300,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>B106:G106</t>
+          <t>B108:G108</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Royice Roberts and Pauline Roberts, JTWROS (1.333200 NMA)</t>
+          <t>TRACT 6 estimated owner: Sara M. Smith — last located record owner; no later conveyance located; current status not confirmed (0.200000 NMA)</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1063/164; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 89/422; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/422. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -3332,12 +3332,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>B107:G107</t>
+          <t>B109:G109</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Sara M. Smith (0.200000 NMA)</t>
+          <t>TRACT 6 estimated owner: Timothy Adrian Godwin — last located record owner; no later conveyance located; current status not confirmed (0.666600 NMA)</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/422; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 1090/95 (face stamp; index reads 96); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1090/95 (face stamp. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -3364,12 +3364,12 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>B108:G108</t>
+          <t>B110:G110</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Timothy Adrian Godwin (0.666600 NMA)</t>
+          <t>TRACT 6 estimated owner: Bettye Folmar Norris — last located record owner; no later conveyance located; current status not confirmed (5.000000 NMA)</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1090/95 (face stamp; index reads 96); EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: DECR 262/490-493 (P-71-473); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 262/490-493 (P-71-473). Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -3396,12 +3396,12 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>B109:G109</t>
+          <t>B115:G115</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>TRACT 6 estimated owner: Bettye Folmar Norris (5.000000 NMA)</t>
+          <t>TRACT 7 estimated owner: C. R. Bennett (812 Palace Building, Tulsa) — last located record owner; no later conveyance located; current status not confirmed (40.000000 NMA)</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 262/490-493 (P-71-473); EST.* Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 81/194; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 81/194. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -3428,12 +3428,12 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>B114:G114</t>
+          <t>B116:G116</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>TRACT 7 estimated owner: C. R. Bennett (812 Palace Building, Tulsa) (40.000000 NMA)</t>
+          <t>TRACT 7 estimated owner: Unresolved successors of S. A. Garrett (last proved record owner) — chain-out not located (35.000000 NMA)</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 81/194; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>ASSUMED: 35.000000 NMA residual vests in last record owner; Garrett chain-out not located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -3460,12 +3460,12 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>B115:G115</t>
+          <t>B117:G117</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>TRACT 7 estimated owner: S. A. Garrett, or his unlocated successors and assigns (35.000000 NMA)</t>
+          <t>TRACT 7 estimated owner: W. F. Palmer (Wichita Falls, TX) — last located record owner; no later conveyance located; current status not confirmed (5.000000 NMA)</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 35.000000 NMA residual vests in last record owner; Garrett chain-out not located. Current status is not confirmed through the report effective date.</t>
+          <t>EST. last located record owner; Vested: MD 92/115; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 92/115. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -3487,32 +3487,32 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Title </t>
+          <t>OGL</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>B116:G116</t>
+          <t>A2:AB2</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>TRACT 7 estimated owner: W. F. Palmer (Wichita Falls, TX) (5.000000 NMA)</t>
+          <t>OGL 63/33 historic lease terms and qualified status</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>V7, V10</t>
+          <t>MT/V7</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 92/115; EST.* Current status is not confirmed through the report effective date.</t>
+          <t>Book/Page 63/33; Img 0353</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Estimated last-located record owner; current vesting and lease status qualified</t>
+          <t>HBP not independently confirmed; assumed potentially effective</t>
         </is>
       </c>
     </row>
@@ -3524,12 +3524,12 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>A2:AB2</t>
+          <t>A3:AB3</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>OGL 63/33 historic lease terms and qualified status</t>
+          <t>OGL 264/345 historic lease terms and qualified status</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -3539,12 +3539,12 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Book/Page 63/33; Img 0353</t>
+          <t>Book/Page 264/345; Imgs 1197-98</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>HBP not independently confirmed; assumed potentially effective</t>
+          <t>HBP not independently confirmed; recital supports assumed effectiveness</t>
         </is>
       </c>
     </row>
@@ -3556,27 +3556,27 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>A3:AB3</t>
+          <t>A4:AB4</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>OGL 264/345 historic lease terms and qualified status</t>
+          <t>OGL 307/31 historic lease terms and qualified status</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>MT/V7</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Book/Page 264/345; Imgs 1197-98</t>
+          <t>Book/Page 307/31; Imgs 1372</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>HBP not independently confirmed; recital supports assumed effectiveness</t>
+          <t>Status not determined; HBP not independently confirmed</t>
         </is>
       </c>
     </row>
@@ -3588,12 +3588,12 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>A4:AB4</t>
+          <t>A5:AB5</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>OGL 307/31 historic lease terms and qualified status</t>
+          <t>OGL 340/302 historic lease terms and qualified status</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Book/Page 307/31; Imgs 1372</t>
+          <t>Book/Page 340/302; Imgs 1522-23</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
@@ -3620,12 +3620,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>A5:AB5</t>
+          <t>A6:AB6</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>OGL 340/302 historic lease terms and qualified status</t>
+          <t>OGL 340/304 historic lease terms and qualified status</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Book/Page 340/302; Imgs 1522-23</t>
+          <t>Book/Page 340/304; Imgs 1524-25</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -3652,12 +3652,12 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>A6:AB6</t>
+          <t>A7:AB7</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>OGL 340/304 historic lease terms and qualified status</t>
+          <t>OGL 340/323 historic lease terms and qualified status</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -3667,7 +3667,7 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Book/Page 340/304; Imgs 1524-25</t>
+          <t>Book/Page 340/323; Imgs 1526-27</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -3684,12 +3684,12 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>A7:AB7</t>
+          <t>A8:AB8</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>OGL 340/323 historic lease terms and qualified status</t>
+          <t>OGL 342/564 historic lease terms and qualified status</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Book/Page 340/323; Imgs 1526-27</t>
+          <t>Book/Page 342/564; Imgs 1542-43</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -3716,12 +3716,12 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>A8:AB8</t>
+          <t>A9:AB9</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>OGL 342/564 historic lease terms and qualified status</t>
+          <t>OGL 342/566 historic lease terms and qualified status</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Book/Page 342/564; Imgs 1542-43</t>
+          <t>Book/Page 342/566; Imgs 1544-45</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -3748,12 +3748,12 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>A9:AB9</t>
+          <t>A10:AB10</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>OGL 342/566 historic lease terms and qualified status</t>
+          <t>OGL 352/719 historic lease terms and qualified status</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Book/Page 342/566; Imgs 1544-45</t>
+          <t>Book/Page 352/719; Imgs 1552-53</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -3780,12 +3780,12 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>A10:AB10</t>
+          <t>A11:AB11</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>OGL 352/719 historic lease terms and qualified status</t>
+          <t>OGL 352/721 historic lease terms and qualified status</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Book/Page 352/719; Imgs 1552-53</t>
+          <t>Book/Page 352/721; Imgs 1554-55</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -3812,12 +3812,12 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>A11:AB11</t>
+          <t>A12:AB12</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>OGL 352/721 historic lease terms and qualified status</t>
+          <t>OGL 376/369 historic lease terms and qualified status</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -3827,7 +3827,7 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Book/Page 352/721; Imgs 1554-55</t>
+          <t>Book/Page 376/369; Imgs 1569-70</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -3844,22 +3844,22 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>A12:AB12</t>
+          <t>A13:AB13</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>OGL 376/369 historic lease terms and qualified status</t>
+          <t>OGL 332/74-75 historic lease terms and qualified status</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>V7</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Book/Page 376/369; Imgs 1569-70</t>
+          <t>Book/Page 332/74-75; Imgs 1457-58</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
@@ -3876,22 +3876,22 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>A13:AB13</t>
+          <t>A14:AB14</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>OGL 332/74-75 historic lease terms and qualified status</t>
+          <t>OGL 341/538 historic lease terms and qualified status</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>V7</t>
+          <t>FV/LC</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Book/Page 332/74-75; Imgs 1457-58</t>
+          <t>Book/Page 341/538; Recited imgs 1568/1812/2031/2300</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -3903,32 +3903,32 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>OGL</t>
+          <t>Runsheet</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>A14:AB14</t>
+          <t>A104:K104</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>OGL 341/538 historic lease terms and qualified status</t>
+          <t>Added missing Section 32 chain lead 1016/7</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>FV/LC</t>
+          <t>V7, V10</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Book/Page 341/538; Recited imgs 1568/1812/2031/2300</t>
+          <t>1016 series; index lead, face not held</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Status not determined; HBP not independently confirmed</t>
+          <t>Locator/qualified evidence; full instrument required</t>
         </is>
       </c>
     </row>
@@ -3940,12 +3940,12 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>A104:K104</t>
+          <t>A105:K105</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Added missing Section 32 chain lead 1016/7</t>
+          <t>Added missing Section 32 chain lead 1016/13</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -3972,12 +3972,12 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>A105:K105</t>
+          <t>A106:K106</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Added missing Section 32 chain lead 1016/13</t>
+          <t>Added missing Section 32 chain lead 1016/18</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -4004,12 +4004,12 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>A106:K106</t>
+          <t>A107:K107</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Added missing Section 32 chain lead 1016/18</t>
+          <t>Added missing Section 32 chain lead 1016/25</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -4036,12 +4036,12 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>A107:K107</t>
+          <t>A108:K108</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Added missing Section 32 chain lead 1016/25</t>
+          <t>Added missing Section 32 chain lead 1016/29</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -4068,12 +4068,12 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>A108:K108</t>
+          <t>A109:K109</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Added missing Section 32 chain lead 1016/29</t>
+          <t>Added missing Section 32 chain lead 1016/33</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -4100,12 +4100,12 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>A109:K109</t>
+          <t>A110:K110</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Added missing Section 32 chain lead 1016/33</t>
+          <t>Added missing Section 32 chain lead 1016/90</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -4132,12 +4132,12 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>A110:K110</t>
+          <t>A111:K111</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Added missing Section 32 chain lead 1016/90</t>
+          <t>Added missing Section 32 chain lead 1697/236</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>1016 series; index lead, face not held</t>
+          <t>Recorded-face lead; required bridge into modern chain</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
@@ -4159,32 +4159,32 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Runsheet</t>
+          <t>Tract 1</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>A111:K111</t>
+          <t>A5:H5</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Added missing Section 32 chain lead 1697/236</t>
+          <t>PAT Patent 3/469 — Sovereign inception; no mineral reservation apparent</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>V7, V10</t>
+          <t>FV, V7, V10, MT</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Recorded-face lead; required bridge into modern chain</t>
+          <t>P-001 / Img 0003</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>Locator/qualified evidence; full instrument required</t>
+          <t>98%</t>
         </is>
       </c>
     </row>
@@ -4196,12 +4196,12 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>A5:H5</t>
+          <t>A6:H6</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>PAT Patent 3/469 — Sovereign inception; no mineral reservation apparent</t>
+          <t>WD Roger Mills 11/214 — NE/4 fee; no reservation apparent</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>P-001 / Img 0003</t>
+          <t>V7 direct-face register</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
@@ -4228,12 +4228,12 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>A6:H6</t>
+          <t>A7:H7</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>WD Roger Mills 11/214 — NE/4 fee; no reservation apparent</t>
+          <t>WD 10/255 — Fee to Adolf; downstream chain incomplete</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -4260,12 +4260,12 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>A7:H7</t>
+          <t>A8:H8</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>WD 10/255 — Fee to Adolf; downstream chain incomplete</t>
+          <t>DECR 83/259 — Collective mineral vesting; allocations require decree</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>V7 direct-face register</t>
+          <t>V7 probate extraction</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
@@ -4292,12 +4292,12 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>A8:H8</t>
+          <t>A9:H9</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>DECR 83/259 — Collective mineral vesting; allocations require decree</t>
+          <t>DECR 845/150-157 — Five 8-NMA estimated last-located interests</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>High quantum / current status open</t>
         </is>
       </c>
     </row>
@@ -4324,12 +4324,12 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>A9:H9</t>
+          <t>A10:H10</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>DECR 845/150-157 — Five 8-NMA estimated last-located interests</t>
+          <t>MD 92/47 — 1.5 NMA each per deed; later one grantee unextracted</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -4339,12 +4339,12 @@
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>V7 probate extraction</t>
+          <t>V7 direct-face register</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>High quantum / current status open</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -4356,12 +4356,12 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>A10:H10</t>
+          <t>A11:H11</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>MD 92/47 — 1.5 NMA each per deed; later one grantee unextracted</t>
+          <t>MD 367/632 — 10 NMA; competing 267/638 out-conveyance must be resolved</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -4376,24 +4376,24 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Tract 1</t>
+          <t>Tract 2</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>A11:H11</t>
+          <t>A5:H5</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>MD 367/632 — 10 NMA; competing 267/638 out-conveyance must be resolved</t>
+          <t>FR Final Receiver Receipt 3894 — Earliest located NW/4 evidence; patent not located</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -4403,12 +4403,12 @@
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>V7 direct-face register</t>
+          <t>P-003 / Img 0005</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>90% identity / 0% patent</t>
         </is>
       </c>
     </row>
@@ -4420,12 +4420,12 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>A5:H5</t>
+          <t>A6:H6</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>FR Final Receiver Receipt 3894 — Earliest located NW/4 evidence; patent not located</t>
+          <t>STIP 153/161-162 — Recorded residual quantum used for estimated ending schedule</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -4435,12 +4435,12 @@
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>P-003 / Img 0005</t>
+          <t>V7 title register</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>90% identity / 0% patent</t>
+          <t>Medium-high</t>
         </is>
       </c>
     </row>
@@ -4452,12 +4452,12 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>A6:H6</t>
+          <t>A7:H7</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>STIP 153/161-162 — Recorded residual quantum used for estimated ending schedule</t>
+          <t>MD/ORDER 85/363-366; 311/817-828 — Estimated last-located mineral interests</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -4472,7 +4472,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>Medium-high</t>
+          <t>Varies; current status open</t>
         </is>
       </c>
     </row>
@@ -4484,12 +4484,12 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>A7:H7</t>
+          <t>A8:H8</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>MD/ORDER 85/363-366; 311/817-828 — Estimated last-located mineral interests</t>
+          <t>DECR P-76-78 — Decree allocation incomplete; 13.333333-NMA residual assumed</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>Varies; current status open</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -4516,12 +4516,12 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>A8:H8</t>
+          <t>A9:H9</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>DECR P-76-78 — Decree allocation incomplete; 13.333333-NMA residual assumed</t>
+          <t>OGL 340/323 — N/2 NW/4 plus N/2 SW/4; no current HBP conclusion</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -4531,29 +4531,29 @@
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>V7 title register</t>
+          <t>Direct face</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High terms / open status</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>Tract 2</t>
+          <t>Tract 3</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>A9:H9</t>
+          <t>A5:H5</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>OGL 340/323 — N/2 NW/4 plus N/2 SW/4; no current HBP conclusion</t>
+          <t>FR Final Receiver Receipt 3895 — Earliest located SW/4 evidence; patent not located</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -4563,12 +4563,12 @@
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>Direct face</t>
+          <t>P-004 / Img 0006</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>High terms / open status</t>
+          <t>90% identity / 0% patent</t>
         </is>
       </c>
     </row>
@@ -4580,12 +4580,12 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>A5:H5</t>
+          <t>A6:H6</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>FR Final Receiver Receipt 3895 — Earliest located SW/4 evidence; patent not located</t>
+          <t>MD 81/194 — 40 NMA in S/2 SW/4 ending schedule</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
@@ -4595,12 +4595,12 @@
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>P-004 / Img 0006</t>
+          <t>V7 title register</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>90% identity / 0% patent</t>
+          <t>Medium; current status open</t>
         </is>
       </c>
     </row>
@@ -4612,12 +4612,12 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>A6:H6</t>
+          <t>A7:H7</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>MD 81/194 — 40 NMA in S/2 SW/4 ending schedule</t>
+          <t>MD/DECR 85/222; 262/490-493 — Estimated last-located interests</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
@@ -4632,7 +4632,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>Medium; current status open</t>
+          <t>Varies</t>
         </is>
       </c>
     </row>
@@ -4644,12 +4644,12 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>A7:H7</t>
+          <t>A8:H8</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>MD/DECR 85/222; 262/490-493 — Estimated last-located interests</t>
+          <t>OGL 340/302; 340/304; 342/564; 342/566 — Overlapping N/2 SW/4 leases; not additive</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
@@ -4659,12 +4659,12 @@
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>V7 title register</t>
+          <t>Direct faces</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>Varies</t>
+          <t>High terms / open status</t>
         </is>
       </c>
     </row>
@@ -4676,12 +4676,12 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>A8:H8</t>
+          <t>A9:H9</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>OGL 340/302; 340/304; 342/564; 342/566 — Overlapping N/2 SW/4 leases; not additive</t>
+          <t>ASG 872/279 — Top Morrow-19,480 ft; ORRIs reserved; modern bridge open</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
@@ -4691,29 +4691,29 @@
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>Direct faces</t>
+          <t>Direct images</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>High terms / open status</t>
+          <t>98% historic / open current</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Tract 3</t>
+          <t>Tract 4</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>A9:H9</t>
+          <t>A5:H5</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>ASG 872/279 — Top Morrow-19,480 ft; ORRIs reserved; modern bridge open</t>
+          <t>FR Final Receiver Receipt — Earliest located SE/4 evidence; Biggs/Bigge patent remains missing</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -4723,12 +4723,12 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>Direct images</t>
+          <t>P-002 / Img 0004</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>98% historic / open current</t>
+          <t>90% identity / 0% patent</t>
         </is>
       </c>
     </row>
@@ -4740,12 +4740,12 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>A5:H5</t>
+          <t>A6:H6</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>FR Final Receiver Receipt — Earliest located SE/4 evidence; Biggs/Bigge patent remains missing</t>
+          <t>OGL 63/33 — E/2 SE/4, 1/8 royalty, 10-year term; present status open</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
@@ -4755,12 +4755,12 @@
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>P-002 / Img 0004</t>
+          <t>Direct face</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>90% identity / 0% patent</t>
+          <t>98% terms</t>
         </is>
       </c>
     </row>
@@ -4772,12 +4772,12 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>A6:H6</t>
+          <t>A7:H7</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>OGL 63/33 — E/2 SE/4, 1/8 royalty, 10-year term; present status open</t>
+          <t>ASG 244/432 — Historic 63/33 assignment branch</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -4787,12 +4787,12 @@
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>Direct face</t>
+          <t>Direct image</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>98% terms</t>
+          <t>96%</t>
         </is>
       </c>
     </row>
@@ -4804,12 +4804,12 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>A7:H7</t>
+          <t>A8:H8</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>ASG 244/432 — Historic 63/33 assignment branch</t>
+          <t>WB ASG 845/47 — Pearl wellbore 11,100-19,480 ft; 1/8 ORRI</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>98% historic</t>
         </is>
       </c>
     </row>
@@ -4836,12 +4836,12 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>A8:H8</t>
+          <t>A9:H9</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>WB ASG 845/47 — Pearl wellbore 11,100-19,480 ft; 1/8 ORRI</t>
+          <t>OGL 307/31 — W/2 SE/4 and S/2 SW/4; present status open</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
@@ -4851,29 +4851,29 @@
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>Direct image</t>
+          <t>Direct face</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>98% historic</t>
+          <t>98% terms</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Tract 4</t>
+          <t>Tract 5</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>A9:H9</t>
+          <t>A5:H5</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>OGL 307/31 — W/2 SE/4 and S/2 SW/4; present status open</t>
+          <t>ASG 1697/236 — Scheduled predecessor lead; full Exhibit A controls</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
@@ -4883,12 +4883,12 @@
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>Direct face</t>
+          <t>Recorded face / Exhibit A required</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>98% terms</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -4900,12 +4900,12 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>A5:H5</t>
+          <t>A6:H6</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>ASG 1697/236 — Scheduled predecessor lead; full Exhibit A controls</t>
+          <t>ASG 2340/490 — Full-section indexed; missing Tapstone/asset bridge schedules</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -4915,12 +4915,12 @@
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>Recorded face / Exhibit A required</t>
+          <t>Index / schedule missing</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High metadata / low scope</t>
         </is>
       </c>
     </row>
@@ -4932,12 +4932,12 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>A6:H6</t>
+          <t>A7:H7</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>ASG 2340/490 — Full-section indexed; missing Tapstone/asset bridge schedules</t>
+          <t>ASG 2371/470-494 — 51.25%/48.75% transaction branches; not current WI</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -4947,12 +4947,12 @@
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>Index / schedule missing</t>
+          <t>Index / instrument partial</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>High metadata / low scope</t>
+          <t>High parties / low asset quantum</t>
         </is>
       </c>
     </row>
@@ -4964,12 +4964,12 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>A7:H7</t>
+          <t>A8:H8</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>ASG 2371/470-494 — 51.25%/48.75% transaction branches; not current WI</t>
+          <t>MERGER 2389/500-580 — Corporate consolidation; asset-specific effect open</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -4979,12 +4979,12 @@
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>Index / instrument partial</t>
+          <t>Index / certificate missing</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>High parties / low asset quantum</t>
+          <t>High metadata</t>
         </is>
       </c>
     </row>
@@ -4996,12 +4996,12 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>A8:H8</t>
+          <t>A9:H9</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>MERGER 2389/500-580 — Corporate consolidation; asset-specific effect open</t>
+          <t>CONV 2395/415-464 — OK48147.001.1 identified; allocation/estate/depth blank</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -5011,12 +5011,12 @@
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>Index / certificate missing</t>
+          <t>Reviewed asset line 2395/462</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>High metadata</t>
+          <t>High asset identity / low quantum</t>
         </is>
       </c>
     </row>
@@ -5028,12 +5028,12 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>A9:H9</t>
+          <t>A10:H10</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>CONV 2395/415-464 — OK48147.001.1 identified; allocation/estate/depth blank</t>
+          <t>CONV 2400/551-567 — Latest supported named claimant; exact current WI/NRI open</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>Reviewed asset line 2395/462</t>
+          <t>Reviewed asset line 2400/566</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
@@ -5060,12 +5060,12 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>A10:H10</t>
+          <t>A11:H11</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>CONV 2400/551-567 — Latest supported named claimant; exact current WI/NRI open</t>
+          <t>AGMT 2476/121-130 — Agreement, not facial conveyance; current vesting effect open</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -5075,44 +5075,44 @@
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>Reviewed asset line 2400/566</t>
+          <t>Index/public metadata</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>High asset identity / low quantum</t>
+          <t>High metadata / low title effect</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Tract 5</t>
+          <t>WI 1</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>A11:H11</t>
+          <t>A5:H5</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>AGMT 2476/121-130 — Agreement, not facial conveyance; current vesting effect open</t>
+          <t>Historic scheduled predecessor lead</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>FV, V7, V10, MT</t>
+          <t>LC, V7, V10, FV</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>Index/public metadata</t>
+          <t>1697/236</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>High metadata / low title effect</t>
+          <t>Full Exhibit A required</t>
         </is>
       </c>
     </row>
@@ -5124,12 +5124,12 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>A5:H5</t>
+          <t>A6:H6</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>Historic scheduled predecessor lead</t>
+          <t>Potential bridge branch</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -5139,12 +5139,12 @@
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>1697/236</t>
+          <t>2340/403</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>Full Exhibit A required</t>
+          <t>Missing Tapstone schedule/bridge</t>
         </is>
       </c>
     </row>
@@ -5156,12 +5156,12 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>A6:H6</t>
+          <t>A7:H7</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>Potential bridge branch</t>
+          <t>Principal indexed predecessor</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -5171,12 +5171,12 @@
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>2340/403</t>
+          <t>2340/490</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>Missing Tapstone schedule/bridge</t>
+          <t>Asset schedule absent</t>
         </is>
       </c>
     </row>
@@ -5188,12 +5188,12 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>A7:H7</t>
+          <t>A8:H8</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>Principal indexed predecessor</t>
+          <t>Keep branches separate</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -5203,12 +5203,12 @@
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>2340/490</t>
+          <t>2371/470-494</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>Asset schedule absent</t>
+          <t>Not current Section 32 WI</t>
         </is>
       </c>
     </row>
@@ -5220,12 +5220,12 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>A8:H8</t>
+          <t>A9:H9</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>Keep branches separate</t>
+          <t>Merger path</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -5235,12 +5235,12 @@
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>2371/470-494</t>
+          <t>2389/500-580</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>Not current Section 32 WI</t>
+          <t>Certificate and schedules absent</t>
         </is>
       </c>
     </row>
@@ -5252,12 +5252,12 @@
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>A9:H9</t>
+          <t>A10:H10</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>Merger path</t>
+          <t>Asset identity supported</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
@@ -5267,12 +5267,12 @@
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>2389/500-580</t>
+          <t>2395/415-464</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>Certificate and schedules absent</t>
+          <t>Estate/depth/quantum blank</t>
         </is>
       </c>
     </row>
@@ -5284,12 +5284,12 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>A10:H10</t>
+          <t>A11:H11</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>Asset identity supported</t>
+          <t>Latest supported named claimant</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -5299,12 +5299,12 @@
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>2395/415-464</t>
+          <t>2400/551-567</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>Estate/depth/quantum blank</t>
+          <t>Later filings and exact quantum open</t>
         </is>
       </c>
     </row>
@@ -5316,12 +5316,12 @@
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>A11:H11</t>
+          <t>A12:H12</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>Latest supported named claimant</t>
+          <t>Later context only</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -5331,44 +5331,44 @@
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>2400/551-567</t>
+          <t>2451/4-23; 2476/121</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>Later filings and exact quantum open</t>
+          <t>Read complete instruments</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>WI 1</t>
+          <t>WI 2</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>A12:H12</t>
+          <t>A5:H5</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>Later context only</t>
+          <t>Historic only; survival open</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>LC, V7, V10, FV</t>
+          <t>FV, V7, V10, MT</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>2451/4-23; 2476/121</t>
+          <t>502/267</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>Read complete instruments</t>
+          <t>Payout, reversion and releases</t>
         </is>
       </c>
     </row>
@@ -5380,12 +5380,12 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>A5:H5</t>
+          <t>A6:H6</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>Historic only; survival open</t>
+          <t>Historic allocation only</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -5395,12 +5395,12 @@
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>502/267</t>
+          <t>509/220</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>Payout, reversion and releases</t>
+          <t>Prove baseline and successors</t>
         </is>
       </c>
     </row>
@@ -5412,12 +5412,12 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>A6:H6</t>
+          <t>A7:H7</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Historic allocation only</t>
+          <t>Historic only; status open</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -5427,12 +5427,12 @@
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>509/220</t>
+          <t>845/47</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>Prove baseline and successors</t>
+          <t>Read unrecorded agreement and releases</t>
         </is>
       </c>
     </row>
@@ -5444,12 +5444,12 @@
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>A7:H7</t>
+          <t>A8:H8</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>Historic only; status open</t>
+          <t>Historic only; bridge open</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -5459,12 +5459,12 @@
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>845/47</t>
+          <t>872/279</t>
         </is>
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>Read unrecorded agreement and releases</t>
+          <t>Complete instrument and 1984 agreement</t>
         </is>
       </c>
     </row>
@@ -5476,12 +5476,12 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>A8:H8</t>
+          <t>A9:H9</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Historic only; bridge open</t>
+          <t>Nemo-dat/source-title defect</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -5491,12 +5491,12 @@
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>872/279</t>
+          <t>1014/75</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>Complete instrument and 1984 agreement</t>
+          <t>Prove assignor WI source</t>
         </is>
       </c>
     </row>
@@ -5508,12 +5508,12 @@
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>A9:H9</t>
+          <t>A10:H10</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>Nemo-dat/source-title defect</t>
+          <t>Separate branch; do not blend</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -5523,12 +5523,12 @@
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>1014/75</t>
+          <t>2183/174; 2185/639</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>Prove assignor WI source</t>
+          <t>Read complete exhibits and legal</t>
         </is>
       </c>
     </row>
@@ -5540,12 +5540,12 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>A10:H10</t>
+          <t>A11:H11</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>Separate branch; do not blend</t>
+          <t>Parallel portfolio branch</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -5555,44 +5555,44 @@
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>2183/174; 2185/639</t>
+          <t>2185/639; 2225/1; 2415/328</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>Read complete exhibits and legal</t>
+          <t>Reconcile Teocalli carve and schedules</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>WI 2</t>
+          <t>Well 1</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>A11:H11</t>
+          <t>A3:Q3</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>Parallel portfolio branch</t>
+          <t>Cora Garrett C-310 / 35-009-00075</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>FV, V7, V10, MT</t>
+          <t>FV official OCC/OTC synthesis; V10 well register</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>2185/639; 2225/1; 2415/328</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>Reconcile Teocalli carve and schedules</t>
+          <t>Operator/status are regulatory context only; lease-specific HBP not independently confirmed</t>
         </is>
       </c>
     </row>
@@ -5604,12 +5604,12 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>A3:Q3</t>
+          <t>A4:Q4</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>Cora Garrett C-310 / 35-009-00075</t>
+          <t>Crook 1-32 / 35-009-20312</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -5619,7 +5619,7 @@
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>No rolling-12-month OTC rows (PUN 009-066620-0-0000, Active, 640 ac, still lists BP). AC/DRY under Complete Oil &amp; Gas Services LLC; Latigo-to-Complete Form 1073MW approved 12/3/2025 (Crook first of 38 wells). AC proves an open wellbore — NOT production or HBP.</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
@@ -5636,12 +5636,12 @@
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>A4:Q4</t>
+          <t>A5:Q5</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>Crook 1-32 / 35-009-20312</t>
+          <t>Pearl 1-32 / 35-009-20605</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -5651,7 +5651,7 @@
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>No rolling-12-month OTC rows (PUN 009-066620-0-0000, Active, 640 ac, still lists BP). AC/DRY under Complete Oil &amp; Gas Services LLC; Latigo-to-Complete Form 1073MW approved 12/3/2025 (Crook first of 38 wells). AC proves an open wellbore — NOT production or HBP.</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="F155" s="2" t="inlineStr">
@@ -5668,12 +5668,12 @@
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>A5:Q5</t>
+          <t>A6:Q6</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>Pearl 1-32 / 35-009-20605</t>
+          <t>Legrand 1-32 / 35-009-20738</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -5700,12 +5700,12 @@
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>A6:Q6</t>
+          <t>A7:Q7</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>Legrand 1-32 / 35-009-20738</t>
+          <t>JGL 1-32 / 35-009-21072</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -5715,7 +5715,7 @@
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>Gas reported 7/2025-4/2026; 4/2026 = 2,367 MCF (OTC PUN 009-101800-0-0000, reported by NextEra Energy Marketing). Production fact only — HBP not concluded.</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
@@ -5732,12 +5732,12 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>A7:Q7</t>
+          <t>A8:Q8</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>JGL 1-32 / 35-009-21072</t>
+          <t>Hanks Crook 1-32 / 35-009-21085</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>Gas reported 7/2025-4/2026; 4/2026 = 2,367 MCF (OTC PUN 009-101800-0-0000, reported by NextEra Energy Marketing). Production fact only — HBP not concluded.</t>
+          <t>Active PUN returned no rolling-12-month rows on 7/9/2026.</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
@@ -5764,12 +5764,12 @@
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>A8:Q8</t>
+          <t>A9:Q9</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>Hanks Crook 1-32 / 35-009-21085</t>
+          <t>Crook-Legrand 1-32 / 35-009-21166</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -5779,7 +5779,7 @@
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>Active PUN returned no rolling-12-month rows on 7/9/2026.</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
@@ -5796,12 +5796,12 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>A9:Q9</t>
+          <t>A10:Q10</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>Crook-Legrand 1-32 / 35-009-21166</t>
+          <t>Legrand 1-32 / 35-009-21236</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -5828,12 +5828,12 @@
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>A10:Q10</t>
+          <t>A11:Q11</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Legrand 1-32 / 35-009-21236</t>
+          <t>Katie 1-32 / 35-009-21245</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -5860,12 +5860,12 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>A11:Q11</t>
+          <t>A12:Q12</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>Katie 1-32 / 35-009-21245</t>
+          <t>Legrand 2-32 / 35-009-21258</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -5892,12 +5892,12 @@
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>A12:Q12</t>
+          <t>A13:Q13</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>Legrand 2-32 / 35-009-21258</t>
+          <t>Twin 1-32 / 35-009-21391</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
@@ -5924,12 +5924,12 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>A13:Q13</t>
+          <t>A14:Q14</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>Twin 1-32 / 35-009-21391</t>
+          <t>Carlson 32-11-25 12H / 35-009-21893</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>Gas through 5/2026; 5/2026 = 2,113 MCF (OTC PUN 009-211663-0-0000, Active, 640 ac). OTC displays API 009-21903 on this PUN — that API belongs to the permit-only Riviera 9H (approved 10/2/2013, expired 4/2/2014); conflict carried. Operator chain per official OCC forms: Linn → EnerVest → BP → Latigo.</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
@@ -5956,12 +5956,12 @@
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>A14:Q14</t>
+          <t>A15:Q15</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>Carlson 32-11-25 12H / 35-009-21893</t>
+          <t>Carlson 32-11-25 7H / 35-009-21923</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
@@ -5971,7 +5971,7 @@
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>Gas through 5/2026; 5/2026 = 2,113 MCF (OTC PUN 009-211663-0-0000, Active, 640 ac). OTC displays API 009-21903 on this PUN — that API belongs to the permit-only Riviera 9H (approved 10/2/2013, expired 4/2/2014); conflict carried. Operator chain per official OCC forms: Linn → EnerVest → BP → Latigo.</t>
+          <t>Historic completion facts only — not proof of current production, lease HBP or title.</t>
         </is>
       </c>
       <c r="F165" s="2" t="inlineStr">
@@ -5988,12 +5988,12 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>A15:Q15</t>
+          <t>A16:Q16</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>Carlson 32-11-25 7H / 35-009-21923</t>
+          <t>Carlson 32-11-25 10H / 35-009-21933</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
@@ -6012,40 +6012,8 @@
         </is>
       </c>
     </row>
-    <row r="167">
-      <c r="A167" s="2" t="inlineStr">
-        <is>
-          <t>Well 1</t>
-        </is>
-      </c>
-      <c r="B167" s="2" t="inlineStr">
-        <is>
-          <t>A16:Q16</t>
-        </is>
-      </c>
-      <c r="C167" s="2" t="inlineStr">
-        <is>
-          <t>Carlson 32-11-25 10H / 35-009-21933</t>
-        </is>
-      </c>
-      <c r="D167" s="2" t="inlineStr">
-        <is>
-          <t>FV official OCC/OTC synthesis; V10 well register</t>
-        </is>
-      </c>
-      <c r="E167" s="2" t="inlineStr">
-        <is>
-          <t>Historic completion facts only — not proof of current production, lease HBP or title.</t>
-        </is>
-      </c>
-      <c r="F167" s="2" t="inlineStr">
-        <is>
-          <t>Operator/status are regulatory context only; lease-specific HBP not independently confirmed</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F167"/>
+  <autoFilter ref="A1:F166"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Regenerate champion with Teocalli qualification
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SECTION32_BEST_OF_BEST_TOURNAMENT_20260806/FINAL_CHAMPION/SECTION32_BEST_OF_BEST_SOURCE_LINEAGE_20260806.xlsx
+++ b/SECTION32_BEST_OF_BEST_TOURNAMENT_20260806/FINAL_CHAMPION/SECTION32_BEST_OF_BEST_SOURCE_LINEAGE_20260806.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Conflict Register" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cell Lineage'!$A$1:$F$166</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cell Lineage'!$A$1:$F$167</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -689,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F166"/>
+  <dimension ref="A1:F167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5289,7 +5289,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>Latest supported named claimant</t>
+          <t>Latest supported named claimant through search cutoff</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -5321,7 +5321,7 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>Later context only</t>
+          <t>Potential post-cutoff divestiture; Section 32 effect unknown</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -5331,44 +5331,44 @@
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>2451/4-23; 2476/121</t>
+          <t>2434/751</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>Read complete instruments</t>
+          <t>Read complete assignment and schedule before calling Diversified current</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>WI 2</t>
+          <t>WI 1</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>A5:H5</t>
+          <t>A13:H13</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>Historic only; survival open</t>
+          <t>Later context only</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>FV, V7, V10, MT</t>
+          <t>LC, V7, V10, FV</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>502/267</t>
+          <t>2451/4-23; 2476/121</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>Payout, reversion and releases</t>
+          <t>Read complete instruments</t>
         </is>
       </c>
     </row>
@@ -5380,12 +5380,12 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>A6:H6</t>
+          <t>A5:H5</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>Historic allocation only</t>
+          <t>Historic only; survival open</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -5395,12 +5395,12 @@
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>509/220</t>
+          <t>502/267</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>Prove baseline and successors</t>
+          <t>Payout, reversion and releases</t>
         </is>
       </c>
     </row>
@@ -5412,12 +5412,12 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>A7:H7</t>
+          <t>A6:H6</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Historic only; status open</t>
+          <t>Historic allocation only</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -5427,12 +5427,12 @@
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>845/47</t>
+          <t>509/220</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>Read unrecorded agreement and releases</t>
+          <t>Prove baseline and successors</t>
         </is>
       </c>
     </row>
@@ -5444,12 +5444,12 @@
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>A8:H8</t>
+          <t>A7:H7</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>Historic only; bridge open</t>
+          <t>Historic only; status open</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -5459,12 +5459,12 @@
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>872/279</t>
+          <t>845/47</t>
         </is>
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>Complete instrument and 1984 agreement</t>
+          <t>Read unrecorded agreement and releases</t>
         </is>
       </c>
     </row>
@@ -5476,12 +5476,12 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>A9:H9</t>
+          <t>A8:H8</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Nemo-dat/source-title defect</t>
+          <t>Historic only; bridge open</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -5491,12 +5491,12 @@
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>1014/75</t>
+          <t>872/279</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>Prove assignor WI source</t>
+          <t>Complete instrument and 1984 agreement</t>
         </is>
       </c>
     </row>
@@ -5508,12 +5508,12 @@
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>A10:H10</t>
+          <t>A9:H9</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>Separate branch; do not blend</t>
+          <t>Nemo-dat/source-title defect</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -5523,12 +5523,12 @@
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>2183/174; 2185/639</t>
+          <t>1014/75</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>Read complete exhibits and legal</t>
+          <t>Prove assignor WI source</t>
         </is>
       </c>
     </row>
@@ -5540,12 +5540,12 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>A11:H11</t>
+          <t>A10:H10</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>Parallel portfolio branch</t>
+          <t>Separate branch; do not blend</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -5555,44 +5555,44 @@
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>2185/639; 2225/1; 2415/328</t>
+          <t>2183/174; 2185/639</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>Reconcile Teocalli carve and schedules</t>
+          <t>Read complete exhibits and legal</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>Well 1</t>
+          <t>WI 2</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>A3:Q3</t>
+          <t>A11:H11</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>Cora Garrett C-310 / 35-009-00075</t>
+          <t>Parallel portfolio branch</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>FV official OCC/OTC synthesis; V10 well register</t>
+          <t>FV, V7, V10, MT</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>2185/639; 2225/1; 2415/328</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>Operator/status are regulatory context only; lease-specific HBP not independently confirmed</t>
+          <t>Reconcile Teocalli carve and schedules</t>
         </is>
       </c>
     </row>
@@ -5604,12 +5604,12 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>A4:Q4</t>
+          <t>A3:Q3</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>Crook 1-32 / 35-009-20312</t>
+          <t>Cora Garrett C-310 / 35-009-00075</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -5619,7 +5619,7 @@
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>No rolling-12-month OTC rows (PUN 009-066620-0-0000, Active, 640 ac, still lists BP). AC/DRY under Complete Oil &amp; Gas Services LLC; Latigo-to-Complete Form 1073MW approved 12/3/2025 (Crook first of 38 wells). AC proves an open wellbore — NOT production or HBP.</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
@@ -5636,12 +5636,12 @@
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>A5:Q5</t>
+          <t>A4:Q4</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>Pearl 1-32 / 35-009-20605</t>
+          <t>Crook 1-32 / 35-009-20312</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -5651,7 +5651,7 @@
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>No rolling-12-month OTC rows (PUN 009-066620-0-0000, Active, 640 ac, still lists BP). AC/DRY under Complete Oil &amp; Gas Services LLC; Latigo-to-Complete Form 1073MW approved 12/3/2025 (Crook first of 38 wells). AC proves an open wellbore — NOT production or HBP.</t>
         </is>
       </c>
       <c r="F155" s="2" t="inlineStr">
@@ -5668,12 +5668,12 @@
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>A6:Q6</t>
+          <t>A5:Q5</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>Legrand 1-32 / 35-009-20738</t>
+          <t>Pearl 1-32 / 35-009-20605</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -5700,12 +5700,12 @@
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>A7:Q7</t>
+          <t>A6:Q6</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>JGL 1-32 / 35-009-21072</t>
+          <t>Legrand 1-32 / 35-009-20738</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -5715,7 +5715,7 @@
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>Gas reported 7/2025-4/2026; 4/2026 = 2,367 MCF (OTC PUN 009-101800-0-0000, reported by NextEra Energy Marketing). Production fact only — HBP not concluded.</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
@@ -5732,12 +5732,12 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>A8:Q8</t>
+          <t>A7:Q7</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>Hanks Crook 1-32 / 35-009-21085</t>
+          <t>JGL 1-32 / 35-009-21072</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>Active PUN returned no rolling-12-month rows on 7/9/2026.</t>
+          <t>Gas reported 7/2025-4/2026; 4/2026 = 2,367 MCF (OTC PUN 009-101800-0-0000, reported by NextEra Energy Marketing). Production fact only — HBP not concluded.</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
@@ -5764,12 +5764,12 @@
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>A9:Q9</t>
+          <t>A8:Q8</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>Crook-Legrand 1-32 / 35-009-21166</t>
+          <t>Hanks Crook 1-32 / 35-009-21085</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -5779,7 +5779,7 @@
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>Active PUN returned no rolling-12-month rows on 7/9/2026.</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
@@ -5796,12 +5796,12 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>A10:Q10</t>
+          <t>A9:Q9</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>Legrand 1-32 / 35-009-21236</t>
+          <t>Crook-Legrand 1-32 / 35-009-21166</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -5828,12 +5828,12 @@
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>A11:Q11</t>
+          <t>A10:Q10</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Katie 1-32 / 35-009-21245</t>
+          <t>Legrand 1-32 / 35-009-21236</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -5860,12 +5860,12 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>A12:Q12</t>
+          <t>A11:Q11</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>Legrand 2-32 / 35-009-21258</t>
+          <t>Katie 1-32 / 35-009-21245</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -5892,12 +5892,12 @@
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>A13:Q13</t>
+          <t>A12:Q12</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>Twin 1-32 / 35-009-21391</t>
+          <t>Legrand 2-32 / 35-009-21258</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
@@ -5924,12 +5924,12 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>A14:Q14</t>
+          <t>A13:Q13</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>Carlson 32-11-25 12H / 35-009-21893</t>
+          <t>Twin 1-32 / 35-009-21391</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>Gas through 5/2026; 5/2026 = 2,113 MCF (OTC PUN 009-211663-0-0000, Active, 640 ac). OTC displays API 009-21903 on this PUN — that API belongs to the permit-only Riviera 9H (approved 10/2/2013, expired 4/2/2014); conflict carried. Operator chain per official OCC forms: Linn → EnerVest → BP → Latigo.</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
@@ -5956,12 +5956,12 @@
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>A15:Q15</t>
+          <t>A14:Q14</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>Carlson 32-11-25 7H / 35-009-21923</t>
+          <t>Carlson 32-11-25 12H / 35-009-21893</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
@@ -5971,7 +5971,7 @@
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>Historic completion facts only — not proof of current production, lease HBP or title.</t>
+          <t>Gas through 5/2026; 5/2026 = 2,113 MCF (OTC PUN 009-211663-0-0000, Active, 640 ac). OTC displays API 009-21903 on this PUN — that API belongs to the permit-only Riviera 9H (approved 10/2/2013, expired 4/2/2014); conflict carried. Operator chain per official OCC forms: Linn → EnerVest → BP → Latigo.</t>
         </is>
       </c>
       <c r="F165" s="2" t="inlineStr">
@@ -5988,32 +5988,64 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
+          <t>A15:Q15</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Carlson 32-11-25 7H / 35-009-21923</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>FV official OCC/OTC synthesis; V10 well register</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>Historic completion facts only — not proof of current production, lease HBP or title.</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>Operator/status are regulatory context only; lease-specific HBP not independently confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>Well 1</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
           <t>A16:Q16</t>
         </is>
       </c>
-      <c r="C166" s="2" t="inlineStr">
+      <c r="C167" s="2" t="inlineStr">
         <is>
           <t>Carlson 32-11-25 10H / 35-009-21933</t>
         </is>
       </c>
-      <c r="D166" s="2" t="inlineStr">
+      <c r="D167" s="2" t="inlineStr">
         <is>
           <t>FV official OCC/OTC synthesis; V10 well register</t>
         </is>
       </c>
-      <c r="E166" s="2" t="inlineStr">
+      <c r="E167" s="2" t="inlineStr">
         <is>
           <t>Historic completion facts only — not proof of current production, lease HBP or title.</t>
         </is>
       </c>
-      <c r="F166" s="2" t="inlineStr">
+      <c r="F167" s="2" t="inlineStr">
         <is>
           <t>Operator/status are regulatory context only; lease-specific HBP not independently confirmed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F166"/>
+  <autoFilter ref="A1:F167"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6286,7 +6318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6647,6 +6679,33 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>C-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Post-cutoff Bk 2434/Pg 751 assigns assets from Diversified/DP Legacy Central to Teocalli, but its schedule is unread.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>V10 current-WI master; post-03/02/2023 index metadata</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Diversified is described only as the latest supported named claimant through Bk 2400/Pg 551-567, subject to this potential later divestiture.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Read the complete 2434/751 assignment and determine whether Section 32 or OK48147.001.1 is included.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Reissue report after final release audit
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SECTION32_BEST_OF_BEST_TOURNAMENT_20260806/FINAL_CHAMPION/SECTION32_BEST_OF_BEST_SOURCE_LINEAGE_20260806.xlsx
+++ b/SECTION32_BEST_OF_BEST_TOURNAMENT_20260806/FINAL_CHAMPION/SECTION32_BEST_OF_BEST_SOURCE_LINEAGE_20260806.xlsx
@@ -755,7 +755,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 65.000000 NMA residual vests in last traced record owner (WD 10/255); no chain-out located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: WD 10/255. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>ASSUMED: 65.000000 NMA residual vests in last traced record owner (WD 10/255); no chain-out located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: WD 10/255. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 92/47; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 92/47. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 92/47; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 92/47. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 367/632; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 367/632. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 367/632; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 367/632. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 250/26; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 250/26. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 250/26; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 250/26. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR 845/150-152 and 845/157; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 845/150-152 and 845/157. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 40.000000 NMA vests collectively per decree; individual allocations not stated on the face. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>ASSUMED: 40.000000 NMA vests collectively per decree; individual allocations not stated on the face. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: holds 1.500000 NMA per the recorded deed; grantee name not extracted from the face. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>ASSUMED: holds 1.500000 NMA per the recorded deed; grantee name not extracted from the face. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: STIPULATION (RECORDED QUANTUM) 153/161-162. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: STIPULATION (RECORDED QUANTUM) 153/161-162. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: STIPULATION (RECORDED QUANTUM) 153/161-162. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: STIPULATION (RECORDED QUANTUM) 153/161-162. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/365 corr. 87/174; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/365 corr. 87/174. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 85/365 corr. 87/174; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/365 corr. 87/174. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1287/42; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1287/42. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 1287/42; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1287/42. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 312/700-704; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 312/700-704. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR 312/700-704; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 312/700-704. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/424; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/424. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/424; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/424. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/363; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/363. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 85/363; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/363. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/245; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/245. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/245; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/245. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1287/42; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1287/42. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 1287/42; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1287/42. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/428; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/428. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/428; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/428. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/426; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/426. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/426; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/426. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/364; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/364. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 85/364; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/364. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: ORDER 311/817-828. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: ORDER 311/817-828. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/366; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/366. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 85/366; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/366. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 88/172; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 88/172. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 88/172; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 88/172. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: ORDER 311/817-828. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: ORDER 311/817-828. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1619,7 +1619,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/87; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/87. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/87; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/87. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/422; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/422. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/422; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/422. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 12.166667 NMA carried in the Farrar fee chain; connecting instrument not located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>ASSUMED: 12.166667 NMA carried in the Farrar fee chain; connecting instrument not located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 6.750000 NMA per 92/468 (index) and later family instruments not read. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: 92/468. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>ASSUMED: 6.750000 NMA per 92/468 (index) and later family instruments not read. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: 92/468. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 86/21; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 86/21. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 86/21; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 86/21. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 13.333333 NMA residue exposed by DECR P-76-78 vests in untraced Keathley successors. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>ASSUMED: 13.333333 NMA residue exposed by DECR P-76-78 vests in untraced Keathley successors. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/36; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/36. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 85/36; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/36. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR P-76-78, pages 349-350 (images 1546-1550); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR P-76-78, pages 349-350 (images 1546-1550). Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR P-76-78, pages 349-350 (images 1546-1550); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR P-76-78, pages 349-350 (images 1546-1550). Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR P-76-78, pages 349-350 (images 1546-1550); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR P-76-78, pages 349-350 (images 1546-1550). Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR P-76-78, pages 349-350 (images 1546-1550); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR P-76-78, pages 349-350 (images 1546-1550). Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 74/63; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 74/63. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 74/63; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 74/63. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR P-76-78, pages 349-350 (images 1546-1550); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR P-76-78, pages 349-350 (images 1546-1550). Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR P-76-78, pages 349-350 (images 1546-1550); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR P-76-78, pages 349-350 (images 1546-1550). Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: STIPULATION (RECORDED QUANTUM) 153/161-162. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: STIPULATION (RECORDED QUANTUM) 153/161-162. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: STIPULATION (RECORDED QUANTUM) 153/161-162. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: STIPULATION (RECORDED QUANTUM) 153/161-162; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: STIPULATION (RECORDED QUANTUM) 153/161-162. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1287/42; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1287/42. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 1287/42; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1287/42. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 312/700-704; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 312/700-704. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR 312/700-704; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 312/700-704. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/424; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/424. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/424; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/424. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 333/239-248; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 333/239-248. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR 333/239-248; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 333/239-248. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 88/174; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 88/174. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 88/174; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 88/174. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1287/42; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1287/42. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 1287/42; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1287/42. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/428; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/428. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/428; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/428. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2259,7 +2259,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/426; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/426. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/426; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/426. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 90/242; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 90/242. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 90/242; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 90/242. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 88/172; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 88/172. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 88/172; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 88/172. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 90/241; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 90/241. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 90/241; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 90/241. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/87; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/87. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/87; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/87. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/422; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/422. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/422; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/422. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 90/153; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 90/153. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 90/153; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 90/153. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/315; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/315. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/315; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/315. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/222; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/222. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 85/222; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/222. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 262/490-493 (P-71-473); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 262/490-493 (P-71-473). Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR 262/490-493 (P-71-473); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 262/490-493 (P-71-473). Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 14.166667 NMA carried in the Stevens chain; connecting instrument not located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>ASSUMED: 14.166667 NMA carried in the Stevens chain; connecting instrument not located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 81/194; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 81/194. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 81/194; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 81/194. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 35.000000 NMA carried in the Stevens chain; connecting instrument not located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>ASSUMED: 35.000000 NMA carried in the Stevens chain; connecting instrument not located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 92/115 (previously mis-cited 92/120); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 92/115 (previously mis-cited 92/120). Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 92/115 (previously mis-cited 92/120); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 92/115 (previously mis-cited 92/120). Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1063/166; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1063/166. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 1063/166; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1063/166. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 27.674000 NMA residual vests in OGL 1 lessors of record; succession untraced. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>ASSUMED: 27.674000 NMA residual vests in OGL 1 lessors of record; succession untraced. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/365 corr. 87/174; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/365 corr. 87/174. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 85/365 corr. 87/174; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/365 corr. 87/174. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -2803,7 +2803,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 312/700-704; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 312/700-704. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR 312/700-704; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 312/700-704. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/424; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/424. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/424; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/424. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/363; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/363. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 85/363; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/363. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/244; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/244. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/244; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/244. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/428; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/428. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/428; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/428. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/426; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/426. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/426; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/426. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1090/94; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1090/94. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 1090/94; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1090/94. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/364; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/364. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 85/364; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/364. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -3059,7 +3059,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: ORDER 311/817-828. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: ORDER 311/817-828. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 85/366; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/366. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 85/366; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 85/366. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 88/172; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 88/172. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 88/172; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 88/172. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1063/164; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1063/164. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 1063/164; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1063/164. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1423/148; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1423/148. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 1423/148; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1423/148. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: ORDER 311/817-828. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: ORDER 311/817-828; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: ORDER 311/817-828. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/87; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/87. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/87; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/87. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1063/164; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1063/164. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 1063/164; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1063/164. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 89/422; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/422. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 89/422; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 89/422. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 1090/95 (face stamp; index reads 96); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1090/95 (face stamp. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 1090/95 (face stamp; index reads 96); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 1090/95 (face stamp. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: DECR 262/490-493 (P-71-473); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 262/490-493 (P-71-473). Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: DECR 262/490-493 (P-71-473); EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: DECR 262/490-493 (P-71-473). Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 81/194; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 81/194. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 81/194; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 81/194. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>ASSUMED: 35.000000 NMA residual vests in last record owner; Garrett chain-out not located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>ASSUMED: 35.000000 NMA residual vests in last record owner; Garrett chain-out not located. V10 STATUS: UNRESOLVED — NOT A PROVED CURRENT OWNER. Vesting/source reference: Not stated on Title row. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>EST. last located record owner; Vested: MD 92/115; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 92/115. Forward record search stops 03/02/2023; current status at 08/06/2026 is not confirmed.</t>
+          <t>EST. last located record owner; Vested: MD 92/115; EST.* V10 STATUS: LATEST LOCATED RECORD OWNER — CURRENT STATUS NOT PROVED. Vesting/source reference: MD 92/115. Complete corpus/face review stops 03/02/2023; later Drive/OCR index-only evidence through Bk 2490/Pg 471 does not confirm current status at 08/06/2026.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Finalize audited Section 32 champion report
Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SECTION32_BEST_OF_BEST_TOURNAMENT_20260806/FINAL_CHAMPION/SECTION32_BEST_OF_BEST_SOURCE_LINEAGE_20260806.xlsx
+++ b/SECTION32_BEST_OF_BEST_TOURNAMENT_20260806/FINAL_CHAMPION/SECTION32_BEST_OF_BEST_SOURCE_LINEAGE_20260806.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Source Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Cell Lineage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Component Selection" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Conflict Register" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cell Lineage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Component Selection" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conflict Register" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cell Lineage'!$A$1:$F$166</definedName>
@@ -6024,13 +6024,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6041,15 +6042,20 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Winning Candidate</t>
+          <t>Contestant Supplier</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Winning Candidate Inputs</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Why Selected</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Merged Additions</t>
         </is>
@@ -6063,15 +6069,20 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>GPT-5-6-SOL</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>FV + V10</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>FV has template parity and strongest controlling qualification</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Effective date, estimated-owner method and cure list from V10</t>
         </is>
@@ -6085,15 +6096,20 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>GPT-5-6-SOL</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>V7 geometry rebuilt in FV style</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Seven fee tracts cover the section and are readable at one-page scale</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Leasehold-overlay warning from MT/LC</t>
         </is>
@@ -6107,15 +6123,20 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>GPT-5-6-SOL</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>V7 + V10</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>V7 has most complete owners/NMA/addresses; V10 identifies present-vesting defects</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>All HBP and current-owner labels qualified</t>
         </is>
@@ -6129,15 +6150,20 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>GPT-5-6-SOL</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
           <t>MT + V7 + FV</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>MT reviewed 11 original faces; V7 adds Viersen; FV/LC adds Minton/Hartman</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Uniform lease-specific status qualifications</t>
         </is>
@@ -6151,15 +6177,20 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
+          <t>GPT-5-6-SOL</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
           <t>FV</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Most complete verified chronology</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Missing 1016 series and 1697/236 leads from V7/V10</t>
         </is>
@@ -6173,15 +6204,20 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>GPT-5-6-SOL</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
           <t>V7 + MT + FV</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Best fee/mineral ending schedules and direct-face chain facts</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Grouped by quarter to preserve 13-tab template</t>
         </is>
@@ -6195,15 +6231,20 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>GPT-5-6-SOL</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
           <t>LC + FV</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Strongest OK48147.001.1 modern chain</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Later corporate filings and missing bridge disclosed</t>
         </is>
@@ -6217,15 +6258,20 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
+          <t>GPT-5-6-SOL</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
           <t>LC + V7/V10</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Strongest Diversified branch sequence and transaction split</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>51.25% expressly not treated as current WI</t>
         </is>
@@ -6239,15 +6285,20 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
+          <t>GPT-5-6-SOL</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
           <t>FV + MT/V7</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Best depth/wellbore burden detail</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Parallel Linn/FourPoint/MNR branches separated</t>
         </is>
@@ -6261,15 +6312,20 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>GPT-5-6-SOL</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>FV</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Strongest official OCC/OTC reconciliation</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>V10 conflict and HBP limitation retained</t>
         </is>

</xml_diff>